<commit_message>
updated lab without crt
</commit_message>
<xml_diff>
--- a/TIME TABLE SAMPLE DATA/LAB.xlsx
+++ b/TIME TABLE SAMPLE DATA/LAB.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5afc8f5c19c83632/Desktop/Timetable/TIME TABLE SAMPLE DATA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ganig\Desktop\Time_Table_\TIME TABLE SAMPLE DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="119" documentId="8_{757FFCFB-9E0B-42BF-A4FD-420F2F59D1B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CE3A883-0D6B-41B1-9BC9-999FA611F3C5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C3ABA9D-3CC3-4CA7-B252-84AAAC807C7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BCF9C078-864F-461E-980E-EDA7976046E4}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BCF9C078-864F-461E-980E-EDA7976046E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="27">
   <si>
     <t>YEAR</t>
   </si>
@@ -108,16 +108,13 @@
     <t>2,3,4</t>
   </si>
   <si>
-    <t>5,6</t>
-  </si>
-  <si>
     <t>1,2,3,4</t>
   </si>
   <si>
     <t>G</t>
   </si>
   <si>
-    <t>T</t>
+    <t>1,2,3</t>
   </si>
 </sst>
 </file>
@@ -176,10 +173,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -499,13 +492,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{762F231F-A71F-4894-BFCC-34A32DE3DF15}">
-  <dimension ref="A1:F90"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F101"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="12.44140625" customWidth="1"/>
+    <col min="3" max="3" width="12.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -525,7 +518,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2</v>
       </c>
@@ -545,7 +538,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -565,7 +558,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2</v>
       </c>
@@ -585,7 +578,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2</v>
       </c>
@@ -605,7 +598,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2</v>
       </c>
@@ -625,7 +618,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>2</v>
       </c>
@@ -645,7 +638,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2</v>
       </c>
@@ -665,7 +658,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>2</v>
       </c>
@@ -685,7 +678,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>2</v>
       </c>
@@ -705,7 +698,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>2</v>
       </c>
@@ -725,7 +718,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>2</v>
       </c>
@@ -745,7 +738,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>2</v>
       </c>
@@ -765,7 +758,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>2</v>
       </c>
@@ -785,7 +778,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>2</v>
       </c>
@@ -805,7 +798,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>2</v>
       </c>
@@ -825,7 +818,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>2</v>
       </c>
@@ -845,7 +838,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>2</v>
       </c>
@@ -865,7 +858,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>2</v>
       </c>
@@ -885,7 +878,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>2</v>
       </c>
@@ -905,7 +898,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>2</v>
       </c>
@@ -925,7 +918,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>2</v>
       </c>
@@ -945,7 +938,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>2</v>
       </c>
@@ -965,7 +958,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>2</v>
       </c>
@@ -985,7 +978,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>2</v>
       </c>
@@ -1005,7 +998,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>2</v>
       </c>
@@ -1025,7 +1018,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>2</v>
       </c>
@@ -1045,7 +1038,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>2</v>
       </c>
@@ -1065,7 +1058,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>2</v>
       </c>
@@ -1085,7 +1078,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>3</v>
       </c>
@@ -1096,16 +1089,16 @@
         <v>7</v>
       </c>
       <c r="D30">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E30" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F30">
         <v>2301</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>3</v>
       </c>
@@ -1116,76 +1109,76 @@
         <v>7</v>
       </c>
       <c r="D31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E31" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F31">
-        <v>2301</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+        <v>2303</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C32">
         <v>7</v>
       </c>
       <c r="D32">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E32" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="F32">
         <v>2301</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>3</v>
       </c>
       <c r="B33" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C33">
         <v>7</v>
       </c>
       <c r="D33">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E33" t="s">
         <v>7</v>
       </c>
       <c r="F33">
-        <v>2302</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+        <v>2303</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C34">
         <v>7</v>
       </c>
       <c r="D34">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E34" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="F34">
         <v>2302</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>2</v>
       </c>
@@ -1199,13 +1192,13 @@
         <v>1</v>
       </c>
       <c r="E35" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F35">
         <v>1109</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>2</v>
       </c>
@@ -1225,7 +1218,7 @@
         <v>1109</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>2</v>
       </c>
@@ -1239,13 +1232,13 @@
         <v>2</v>
       </c>
       <c r="E37" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F37">
         <v>1109</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>2</v>
       </c>
@@ -1265,7 +1258,7 @@
         <v>1109</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>2</v>
       </c>
@@ -1285,7 +1278,7 @@
         <v>1109</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>2</v>
       </c>
@@ -1305,7 +1298,7 @@
         <v>1109</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>2</v>
       </c>
@@ -1319,13 +1312,13 @@
         <v>4</v>
       </c>
       <c r="E41" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F41">
         <v>1109</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>2</v>
       </c>
@@ -1345,7 +1338,7 @@
         <v>1109</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>2</v>
       </c>
@@ -1359,13 +1352,13 @@
         <v>6</v>
       </c>
       <c r="E43" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F43">
         <v>1109</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>2</v>
       </c>
@@ -1385,7 +1378,7 @@
         <v>1110</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>2</v>
       </c>
@@ -1405,7 +1398,7 @@
         <v>1110</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>2</v>
       </c>
@@ -1425,7 +1418,7 @@
         <v>1110</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>2</v>
       </c>
@@ -1445,7 +1438,7 @@
         <v>1110</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>2</v>
       </c>
@@ -1465,7 +1458,7 @@
         <v>1110</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>2</v>
       </c>
@@ -1485,7 +1478,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>2</v>
       </c>
@@ -1505,7 +1498,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>2</v>
       </c>
@@ -1525,7 +1518,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>2</v>
       </c>
@@ -1545,7 +1538,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>2</v>
       </c>
@@ -1565,7 +1558,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>2</v>
       </c>
@@ -1585,7 +1578,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>2</v>
       </c>
@@ -1605,7 +1598,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>2</v>
       </c>
@@ -1625,7 +1618,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>2</v>
       </c>
@@ -1645,7 +1638,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>2</v>
       </c>
@@ -1665,7 +1658,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>2</v>
       </c>
@@ -1685,7 +1678,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>2</v>
       </c>
@@ -1705,7 +1698,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>2</v>
       </c>
@@ -1725,7 +1718,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>2</v>
       </c>
@@ -1745,7 +1738,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>2</v>
       </c>
@@ -1762,10 +1755,10 @@
         <v>11</v>
       </c>
       <c r="F63" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>2</v>
       </c>
@@ -1782,10 +1775,10 @@
         <v>11</v>
       </c>
       <c r="F64" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>2</v>
       </c>
@@ -1802,10 +1795,10 @@
         <v>11</v>
       </c>
       <c r="F65" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>2</v>
       </c>
@@ -1822,10 +1815,10 @@
         <v>11</v>
       </c>
       <c r="F66" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>2</v>
       </c>
@@ -1842,10 +1835,10 @@
         <v>11</v>
       </c>
       <c r="F67" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>2</v>
       </c>
@@ -1862,10 +1855,10 @@
         <v>11</v>
       </c>
       <c r="F68" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>2</v>
       </c>
@@ -1882,10 +1875,10 @@
         <v>11</v>
       </c>
       <c r="F69" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>2</v>
       </c>
@@ -1902,10 +1895,10 @@
         <v>11</v>
       </c>
       <c r="F70" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>2</v>
       </c>
@@ -1922,10 +1915,10 @@
         <v>11</v>
       </c>
       <c r="F71" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>2</v>
       </c>
@@ -1942,10 +1935,10 @@
         <v>11</v>
       </c>
       <c r="F72" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>2</v>
       </c>
@@ -1962,10 +1955,10 @@
         <v>11</v>
       </c>
       <c r="F73" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>3</v>
       </c>
@@ -1973,19 +1966,19 @@
         <v>10</v>
       </c>
       <c r="C74">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D74">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E74" t="s">
-        <v>25</v>
-      </c>
-      <c r="F74" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="F74">
+        <v>2303</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>3</v>
       </c>
@@ -1993,19 +1986,19 @@
         <v>10</v>
       </c>
       <c r="C75">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D75">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E75" t="s">
-        <v>25</v>
-      </c>
-      <c r="F75" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="F75">
+        <v>2303</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>3</v>
       </c>
@@ -2013,19 +2006,19 @@
         <v>10</v>
       </c>
       <c r="C76">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D76">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E76" t="s">
-        <v>7</v>
-      </c>
-      <c r="F76" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="F76">
+        <v>2303</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>3</v>
       </c>
@@ -2033,19 +2026,19 @@
         <v>6</v>
       </c>
       <c r="C77">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D77">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E77" t="s">
-        <v>24</v>
-      </c>
-      <c r="F77" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="F77">
+        <v>2301</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>3</v>
       </c>
@@ -2053,19 +2046,19 @@
         <v>6</v>
       </c>
       <c r="C78">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D78">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E78" t="s">
         <v>17</v>
       </c>
-      <c r="F78" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F78">
+        <v>2301</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>3</v>
       </c>
@@ -2073,7 +2066,7 @@
         <v>6</v>
       </c>
       <c r="C79">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D79">
         <v>6</v>
@@ -2081,31 +2074,31 @@
       <c r="E79" t="s">
         <v>17</v>
       </c>
-      <c r="F79" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F79">
+        <v>2301</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>3</v>
       </c>
       <c r="B80" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C80">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D80">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E80" t="s">
-        <v>9</v>
-      </c>
-      <c r="F80" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="F80">
+        <v>2302</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>3</v>
       </c>
@@ -2113,19 +2106,19 @@
         <v>14</v>
       </c>
       <c r="C81">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D81">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E81" t="s">
-        <v>24</v>
-      </c>
-      <c r="F81" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="F81">
+        <v>2302</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>3</v>
       </c>
@@ -2133,59 +2126,59 @@
         <v>14</v>
       </c>
       <c r="C82">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D82">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E82" t="s">
         <v>17</v>
       </c>
-      <c r="F82" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F82">
+        <v>2302</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>3</v>
       </c>
       <c r="B83" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C83">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D83">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E83" t="s">
         <v>17</v>
       </c>
-      <c r="F83" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F83">
+        <v>2301</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>3</v>
       </c>
       <c r="B84" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C84">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D84">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E84" t="s">
-        <v>9</v>
-      </c>
-      <c r="F84" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="F84">
+        <v>2301</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>3</v>
       </c>
@@ -2193,59 +2186,59 @@
         <v>13</v>
       </c>
       <c r="C85">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D85">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E85" t="s">
-        <v>7</v>
-      </c>
-      <c r="F85" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="F85">
+        <v>2301</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>3</v>
       </c>
       <c r="B86" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C86">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D86">
         <v>4</v>
       </c>
       <c r="E86" t="s">
-        <v>25</v>
-      </c>
-      <c r="F86" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="F86">
+        <v>2302</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>3</v>
       </c>
       <c r="B87" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C87">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D87">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E87" t="s">
-        <v>25</v>
-      </c>
-      <c r="F87" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="F87">
+        <v>2302</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>3</v>
       </c>
@@ -2253,56 +2246,276 @@
         <v>12</v>
       </c>
       <c r="C88">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D88">
+        <v>6</v>
+      </c>
+      <c r="E88" t="s">
+        <v>17</v>
+      </c>
+      <c r="F88">
+        <v>2302</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A89">
+        <v>3</v>
+      </c>
+      <c r="B89" t="s">
+        <v>10</v>
+      </c>
+      <c r="C89">
+        <v>20</v>
+      </c>
+      <c r="D89">
         <v>1</v>
       </c>
-      <c r="E88" t="s">
-        <v>7</v>
-      </c>
-      <c r="F88" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89">
-        <v>3</v>
-      </c>
-      <c r="B89" t="s">
+      <c r="E89" t="s">
+        <v>7</v>
+      </c>
+      <c r="F89">
+        <v>2302</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A90">
+        <v>3</v>
+      </c>
+      <c r="B90" t="s">
+        <v>6</v>
+      </c>
+      <c r="C90">
+        <v>20</v>
+      </c>
+      <c r="D90">
+        <v>1</v>
+      </c>
+      <c r="E90" t="s">
+        <v>9</v>
+      </c>
+      <c r="F90">
+        <v>2303</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A91">
+        <v>3</v>
+      </c>
+      <c r="B91" t="s">
+        <v>14</v>
+      </c>
+      <c r="C91">
+        <v>20</v>
+      </c>
+      <c r="D91">
+        <v>2</v>
+      </c>
+      <c r="E91" t="s">
+        <v>7</v>
+      </c>
+      <c r="F91">
+        <v>2302</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A92">
+        <v>3</v>
+      </c>
+      <c r="B92" t="s">
+        <v>13</v>
+      </c>
+      <c r="C92">
+        <v>20</v>
+      </c>
+      <c r="D92">
+        <v>5</v>
+      </c>
+      <c r="E92" t="s">
+        <v>9</v>
+      </c>
+      <c r="F92">
+        <v>2302</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A93">
+        <v>3</v>
+      </c>
+      <c r="B93" t="s">
         <v>12</v>
       </c>
-      <c r="C89">
-        <v>21</v>
-      </c>
-      <c r="D89">
+      <c r="C93">
+        <v>20</v>
+      </c>
+      <c r="D93">
         <v>4</v>
       </c>
-      <c r="E89" t="s">
-        <v>25</v>
-      </c>
-      <c r="F89" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90">
-        <v>3</v>
-      </c>
-      <c r="B90" t="s">
-        <v>12</v>
-      </c>
-      <c r="C90">
-        <v>21</v>
-      </c>
-      <c r="D90">
+      <c r="E93" t="s">
+        <v>7</v>
+      </c>
+      <c r="F93">
+        <v>2302</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A94">
+        <v>3</v>
+      </c>
+      <c r="B94" t="s">
+        <v>20</v>
+      </c>
+      <c r="C94">
+        <v>20</v>
+      </c>
+      <c r="D94">
+        <v>2</v>
+      </c>
+      <c r="E94" t="s">
+        <v>7</v>
+      </c>
+      <c r="F94">
+        <v>2303</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A95">
+        <v>3</v>
+      </c>
+      <c r="B95" t="s">
+        <v>15</v>
+      </c>
+      <c r="C95">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>4</v>
+      </c>
+      <c r="E95" t="s">
+        <v>9</v>
+      </c>
+      <c r="F95">
+        <v>2301</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A96">
+        <v>3</v>
+      </c>
+      <c r="B96" t="s">
+        <v>20</v>
+      </c>
+      <c r="C96">
+        <v>17</v>
+      </c>
+      <c r="D96">
+        <v>4</v>
+      </c>
+      <c r="E96" t="s">
+        <v>26</v>
+      </c>
+      <c r="F96">
+        <v>2303</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A97">
+        <v>3</v>
+      </c>
+      <c r="B97" t="s">
+        <v>20</v>
+      </c>
+      <c r="C97">
+        <v>18</v>
+      </c>
+      <c r="D97">
+        <v>5</v>
+      </c>
+      <c r="E97" t="s">
+        <v>17</v>
+      </c>
+      <c r="F97">
+        <v>2303</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A98">
+        <v>3</v>
+      </c>
+      <c r="B98" t="s">
+        <v>20</v>
+      </c>
+      <c r="C98">
+        <v>19</v>
+      </c>
+      <c r="D98">
         <v>6</v>
       </c>
-      <c r="E90" t="s">
-        <v>25</v>
-      </c>
-      <c r="F90" t="s">
-        <v>27</v>
+      <c r="E98" t="s">
+        <v>17</v>
+      </c>
+      <c r="F98">
+        <v>2303</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A99">
+        <v>3</v>
+      </c>
+      <c r="B99" t="s">
+        <v>15</v>
+      </c>
+      <c r="C99">
+        <v>17</v>
+      </c>
+      <c r="D99">
+        <v>1</v>
+      </c>
+      <c r="E99" t="s">
+        <v>26</v>
+      </c>
+      <c r="F99">
+        <v>2301</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A100">
+        <v>3</v>
+      </c>
+      <c r="B100" t="s">
+        <v>15</v>
+      </c>
+      <c r="C100">
+        <v>18</v>
+      </c>
+      <c r="D100">
+        <v>2</v>
+      </c>
+      <c r="E100" t="s">
+        <v>23</v>
+      </c>
+      <c r="F100">
+        <v>2301</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A101">
+        <v>3</v>
+      </c>
+      <c r="B101" t="s">
+        <v>15</v>
+      </c>
+      <c r="C101">
+        <v>19</v>
+      </c>
+      <c r="D101">
+        <v>3</v>
+      </c>
+      <c r="E101" t="s">
+        <v>26</v>
+      </c>
+      <c r="F101">
+        <v>2301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
time table generation with minor changes
</commit_message>
<xml_diff>
--- a/TIME TABLE SAMPLE DATA/LAB.xlsx
+++ b/TIME TABLE SAMPLE DATA/LAB.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ganig\Desktop\Time_Table_\TIME TABLE SAMPLE DATA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajas\OneDrive\Desktop\Timetable\TIME TABLE SAMPLE DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0D102E7-BD8E-4823-8A7D-0B6A78906159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C785179B-C7D6-42C7-9F76-C1A75874E627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BCF9C078-864F-461E-980E-EDA7976046E4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BCF9C078-864F-461E-980E-EDA7976046E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -105,10 +105,10 @@
     <t>2,3,4</t>
   </si>
   <si>
-    <t>G</t>
-  </si>
-  <si>
     <t>1,2,3</t>
+  </si>
+  <si>
+    <t>GROUND</t>
   </si>
 </sst>
 </file>
@@ -487,12 +487,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{762F231F-A71F-4894-BFCC-34A32DE3DF15}">
   <dimension ref="A1:F85"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="12.453125" customWidth="1"/>
+    <col min="3" max="3" width="12.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -512,7 +512,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>
@@ -532,7 +532,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -552,7 +552,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -572,7 +572,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2</v>
       </c>
@@ -592,7 +592,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2</v>
       </c>
@@ -612,7 +612,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2</v>
       </c>
@@ -632,7 +632,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2</v>
       </c>
@@ -652,7 +652,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2</v>
       </c>
@@ -672,7 +672,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2</v>
       </c>
@@ -692,7 +692,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2</v>
       </c>
@@ -712,7 +712,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2</v>
       </c>
@@ -732,7 +732,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2</v>
       </c>
@@ -752,7 +752,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2</v>
       </c>
@@ -772,7 +772,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2</v>
       </c>
@@ -792,7 +792,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2</v>
       </c>
@@ -812,7 +812,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2</v>
       </c>
@@ -832,7 +832,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2</v>
       </c>
@@ -852,7 +852,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2</v>
       </c>
@@ -872,7 +872,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2</v>
       </c>
@@ -892,7 +892,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>2</v>
       </c>
@@ -912,7 +912,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>2</v>
       </c>
@@ -932,7 +932,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>2</v>
       </c>
@@ -952,7 +952,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>2</v>
       </c>
@@ -972,7 +972,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>2</v>
       </c>
@@ -992,7 +992,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>2</v>
       </c>
@@ -1012,7 +1012,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>2</v>
       </c>
@@ -1032,7 +1032,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>2</v>
       </c>
@@ -1052,7 +1052,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>2</v>
       </c>
@@ -1072,7 +1072,7 @@
         <v>2202</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>3</v>
       </c>
@@ -1092,7 +1092,7 @@
         <v>2301</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>3</v>
       </c>
@@ -1112,7 +1112,7 @@
         <v>2303</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>3</v>
       </c>
@@ -1132,7 +1132,7 @@
         <v>2301</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>3</v>
       </c>
@@ -1152,7 +1152,7 @@
         <v>2303</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>3</v>
       </c>
@@ -1172,7 +1172,7 @@
         <v>2302</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>2</v>
       </c>
@@ -1192,7 +1192,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>2</v>
       </c>
@@ -1212,7 +1212,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>2</v>
       </c>
@@ -1232,7 +1232,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>2</v>
       </c>
@@ -1252,7 +1252,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>2</v>
       </c>
@@ -1272,7 +1272,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>2</v>
       </c>
@@ -1292,7 +1292,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>2</v>
       </c>
@@ -1312,7 +1312,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>2</v>
       </c>
@@ -1332,7 +1332,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>2</v>
       </c>
@@ -1352,7 +1352,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>2</v>
       </c>
@@ -1372,7 +1372,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>2</v>
       </c>
@@ -1392,7 +1392,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>2</v>
       </c>
@@ -1412,7 +1412,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>2</v>
       </c>
@@ -1420,7 +1420,7 @@
         <v>10</v>
       </c>
       <c r="C47">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D47">
         <v>5</v>
@@ -1429,10 +1429,10 @@
         <v>11</v>
       </c>
       <c r="F47" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>2</v>
       </c>
@@ -1440,7 +1440,7 @@
         <v>6</v>
       </c>
       <c r="C48">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D48">
         <v>5</v>
@@ -1449,10 +1449,10 @@
         <v>11</v>
       </c>
       <c r="F48" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>2</v>
       </c>
@@ -1460,7 +1460,7 @@
         <v>14</v>
       </c>
       <c r="C49">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D49">
         <v>5</v>
@@ -1469,10 +1469,10 @@
         <v>11</v>
       </c>
       <c r="F49" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>2</v>
       </c>
@@ -1480,7 +1480,7 @@
         <v>13</v>
       </c>
       <c r="C50">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D50">
         <v>5</v>
@@ -1489,10 +1489,10 @@
         <v>11</v>
       </c>
       <c r="F50" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>2</v>
       </c>
@@ -1500,7 +1500,7 @@
         <v>12</v>
       </c>
       <c r="C51">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D51">
         <v>5</v>
@@ -1509,10 +1509,10 @@
         <v>11</v>
       </c>
       <c r="F51" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>2</v>
       </c>
@@ -1520,7 +1520,7 @@
         <v>16</v>
       </c>
       <c r="C52">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D52">
         <v>5</v>
@@ -1529,10 +1529,10 @@
         <v>11</v>
       </c>
       <c r="F52" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>2</v>
       </c>
@@ -1540,7 +1540,7 @@
         <v>8</v>
       </c>
       <c r="C53">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D53">
         <v>5</v>
@@ -1549,10 +1549,10 @@
         <v>11</v>
       </c>
       <c r="F53" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>2</v>
       </c>
@@ -1560,7 +1560,7 @@
         <v>19</v>
       </c>
       <c r="C54">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D54">
         <v>5</v>
@@ -1569,10 +1569,10 @@
         <v>11</v>
       </c>
       <c r="F54" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>2</v>
       </c>
@@ -1580,7 +1580,7 @@
         <v>15</v>
       </c>
       <c r="C55">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D55">
         <v>5</v>
@@ -1589,10 +1589,10 @@
         <v>11</v>
       </c>
       <c r="F55" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>2</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>21</v>
       </c>
       <c r="C56">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D56">
         <v>5</v>
@@ -1609,10 +1609,10 @@
         <v>11</v>
       </c>
       <c r="F56" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>2</v>
       </c>
@@ -1620,7 +1620,7 @@
         <v>20</v>
       </c>
       <c r="C57">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D57">
         <v>5</v>
@@ -1629,10 +1629,10 @@
         <v>11</v>
       </c>
       <c r="F57" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>3</v>
       </c>
@@ -1652,7 +1652,7 @@
         <v>2303</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>3</v>
       </c>
@@ -1672,7 +1672,7 @@
         <v>2303</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>3</v>
       </c>
@@ -1692,7 +1692,7 @@
         <v>2303</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>3</v>
       </c>
@@ -1712,7 +1712,7 @@
         <v>2301</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>3</v>
       </c>
@@ -1732,7 +1732,7 @@
         <v>2301</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>3</v>
       </c>
@@ -1752,7 +1752,7 @@
         <v>2301</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>3</v>
       </c>
@@ -1772,7 +1772,7 @@
         <v>2302</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>3</v>
       </c>
@@ -1792,7 +1792,7 @@
         <v>2302</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>3</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>2302</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>3</v>
       </c>
@@ -1832,7 +1832,7 @@
         <v>2301</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>3</v>
       </c>
@@ -1852,7 +1852,7 @@
         <v>2301</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>3</v>
       </c>
@@ -1872,7 +1872,7 @@
         <v>2301</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>3</v>
       </c>
@@ -1892,7 +1892,7 @@
         <v>2302</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>3</v>
       </c>
@@ -1912,7 +1912,7 @@
         <v>2302</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>3</v>
       </c>
@@ -1932,7 +1932,7 @@
         <v>2302</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>3</v>
       </c>
@@ -1952,7 +1952,7 @@
         <v>2302</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>3</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>2303</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>3</v>
       </c>
@@ -1992,7 +1992,7 @@
         <v>2302</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>3</v>
       </c>
@@ -2012,7 +2012,7 @@
         <v>2302</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>3</v>
       </c>
@@ -2032,7 +2032,7 @@
         <v>2302</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>3</v>
       </c>
@@ -2052,7 +2052,7 @@
         <v>2303</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>3</v>
       </c>
@@ -2072,7 +2072,7 @@
         <v>2301</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>3</v>
       </c>
@@ -2086,13 +2086,13 @@
         <v>4</v>
       </c>
       <c r="E80" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F80">
         <v>2303</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>3</v>
       </c>
@@ -2112,7 +2112,7 @@
         <v>2303</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>3</v>
       </c>
@@ -2132,7 +2132,7 @@
         <v>2303</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>3</v>
       </c>
@@ -2146,13 +2146,13 @@
         <v>1</v>
       </c>
       <c r="E83" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F83">
         <v>2301</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>3</v>
       </c>
@@ -2172,7 +2172,7 @@
         <v>2301</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>3</v>
       </c>
@@ -2186,7 +2186,7 @@
         <v>3</v>
       </c>
       <c r="E85" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F85">
         <v>2301</v>

</xml_diff>